<commit_message>
Fix table alignment in 28-day months, sync year/month pickers, enable live dynamic yearly & vault metrics, and correct CSS/Excel formulas
</commit_message>
<xml_diff>
--- a/Istiqamah_Tracker_2026_2036.xlsx
+++ b/Istiqamah_Tracker_2026_2036.xlsx
@@ -143,10 +143,13 @@
       <sz val="12"/>
     </font>
     <font>
+      <name val="Calibri"/>
       <b val="1"/>
-      <sz val="8"/>
+      <color rgb="00059669"/>
+      <sz val="9"/>
     </font>
     <font>
+      <b val="1"/>
       <sz val="8"/>
     </font>
     <font>
@@ -465,18 +468,18 @@
     <xf numFmtId="0" fontId="19" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="22" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="14" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="23" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="9" fontId="23" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="24" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="13" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1722,7 +1725,7 @@
         </is>
       </c>
       <c r="D11" s="30">
-        <f>SUM(H35:AP35)</f>
+        <f>SUM(H35:AP35)+SUM(M43:M48)+SUM(H52:H56)</f>
         <v/>
       </c>
     </row>
@@ -3910,7 +3913,7 @@
     </row>
     <row r="38">
       <c r="B38" s="62">
-        <f>SUM(H35:AP35)</f>
+        <f>SUM(H35:AP35)+SUM(M43:M48)+SUM(H52:H56)</f>
         <v/>
       </c>
     </row>
@@ -3965,6 +3968,11 @@
           <t>Wk 5</t>
         </is>
       </c>
+      <c r="M42" s="63" t="inlineStr">
+        <is>
+          <t>Earned ($)</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="50" t="inlineStr">
@@ -3987,6 +3995,10 @@
       <c r="K43" s="49" t="b">
         <v>0</v>
       </c>
+      <c r="M43" s="69">
+        <f>COUNTIF(G43:K43, TRUE)*10.0</f>
+        <v/>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="50" t="inlineStr">
@@ -4009,6 +4021,10 @@
       <c r="K44" s="49" t="b">
         <v>0</v>
       </c>
+      <c r="M44" s="69">
+        <f>COUNTIF(G44:K44, TRUE)*5.0</f>
+        <v/>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="48" t="inlineStr">
@@ -4031,6 +4047,10 @@
       <c r="K45" s="49" t="b">
         <v>0</v>
       </c>
+      <c r="M45" s="69">
+        <f>COUNTIF(G45:K45, TRUE)*5.0</f>
+        <v/>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="51" t="inlineStr">
@@ -4053,6 +4073,10 @@
       <c r="K46" s="49" t="b">
         <v>0</v>
       </c>
+      <c r="M46" s="69">
+        <f>COUNTIF(G46:K46, TRUE)*5.0</f>
+        <v/>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="48" t="inlineStr">
@@ -4075,6 +4099,10 @@
       <c r="K47" s="49" t="b">
         <v>0</v>
       </c>
+      <c r="M47" s="69">
+        <f>COUNTIF(G47:K47, TRUE)*5.0</f>
+        <v/>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="52" t="inlineStr">
@@ -4096,6 +4124,10 @@
       </c>
       <c r="K48" s="49" t="b">
         <v>0</v>
+      </c>
+      <c r="M48" s="69">
+        <f>COUNTIF(G48:K48, TRUE)*5.0</f>
+        <v/>
       </c>
     </row>
     <row r="51" ht="24" customHeight="1">
@@ -4127,6 +4159,10 @@
       <c r="G52" s="49" t="b">
         <v>0</v>
       </c>
+      <c r="H52" s="69">
+        <f>IF(G52=TRUE, 20.0, 0)</f>
+        <v/>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="52" t="inlineStr">
@@ -4137,6 +4173,10 @@
       <c r="G53" s="49" t="b">
         <v>0</v>
       </c>
+      <c r="H53" s="69">
+        <f>IF(G53=TRUE, 25.0, 0)</f>
+        <v/>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="50" t="inlineStr">
@@ -4147,6 +4187,10 @@
       <c r="G54" s="49" t="b">
         <v>0</v>
       </c>
+      <c r="H54" s="69">
+        <f>IF(G54=TRUE, 15.0, 0)</f>
+        <v/>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="52" t="inlineStr">
@@ -4157,6 +4201,10 @@
       <c r="G55" s="49" t="b">
         <v>0</v>
       </c>
+      <c r="H55" s="69">
+        <f>IF(G55=TRUE, 15.0, 0)</f>
+        <v/>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="51" t="inlineStr">
@@ -4166,6 +4214,10 @@
       </c>
       <c r="G56" s="49" t="b">
         <v>0</v>
+      </c>
+      <c r="H56" s="69">
+        <f>IF(G56=TRUE, 10.0, 0)</f>
+        <v/>
       </c>
     </row>
   </sheetData>
@@ -4326,10 +4378,9 @@
           <t>Complete to date (%):</t>
         </is>
       </c>
-      <c r="D9" s="69" t="inlineStr">
-        <is>
-          <t>18%</t>
-        </is>
+      <c r="D9" s="29">
+        <f>AVERAGE(D16,D19,D22,D25,D28,D31,D34,D37,D40,D43,D46,D49)</f>
+        <v/>
       </c>
     </row>
     <row r="11">
@@ -4338,10 +4389,9 @@
           <t>Total earned to date ($):</t>
         </is>
       </c>
-      <c r="D11" s="70" t="inlineStr">
-        <is>
-          <t>$1,752.00</t>
-        </is>
+      <c r="D11" s="30">
+        <f>SUM(K16,K19,K22,K25,K28,K31,K34,K37,K40,K43,K46,K49)</f>
+        <v/>
       </c>
     </row>
     <row r="13" ht="24" customHeight="1">
@@ -4352,327 +4402,305 @@
       </c>
     </row>
     <row r="15" ht="20" customHeight="1">
-      <c r="A15" s="71" t="inlineStr">
+      <c r="A15" s="70" t="inlineStr">
         <is>
           <t>JANUARY</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="B16" s="72" t="inlineStr">
+      <c r="B16" s="71" t="inlineStr">
         <is>
           <t>Completion:</t>
         </is>
       </c>
-      <c r="D16" s="73" t="inlineStr">
-        <is>
-          <t>24%</t>
-        </is>
-      </c>
-      <c r="H16" s="72" t="inlineStr">
+      <c r="D16" s="72" t="n">
+        <v>0</v>
+      </c>
+      <c r="H16" s="71" t="inlineStr">
         <is>
           <t>Total Rewards:</t>
         </is>
       </c>
-      <c r="K16" s="74" t="n">
-        <v>516.5</v>
+      <c r="K16" s="73" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="18" ht="20" customHeight="1">
-      <c r="A18" s="71" t="inlineStr">
+      <c r="A18" s="70" t="inlineStr">
         <is>
           <t>FEBRUARY</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="B19" s="72" t="inlineStr">
+      <c r="B19" s="71" t="inlineStr">
         <is>
           <t>Completion:</t>
         </is>
       </c>
-      <c r="D19" s="73" t="inlineStr">
-        <is>
-          <t>24%</t>
-        </is>
-      </c>
-      <c r="H19" s="72" t="inlineStr">
+      <c r="D19" s="72" t="n">
+        <v>0</v>
+      </c>
+      <c r="H19" s="71" t="inlineStr">
         <is>
           <t>Total Rewards:</t>
         </is>
       </c>
-      <c r="K19" s="74" t="n">
-        <v>516.5</v>
+      <c r="K19" s="73" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="21" ht="20" customHeight="1">
-      <c r="A21" s="71" t="inlineStr">
+      <c r="A21" s="70" t="inlineStr">
         <is>
           <t>MARCH</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="B22" s="72" t="inlineStr">
+      <c r="B22" s="71" t="inlineStr">
         <is>
           <t>Completion:</t>
         </is>
       </c>
-      <c r="D22" s="73" t="inlineStr">
-        <is>
-          <t>24%</t>
-        </is>
-      </c>
-      <c r="H22" s="72" t="inlineStr">
+      <c r="D22" s="72" t="n">
+        <v>0</v>
+      </c>
+      <c r="H22" s="71" t="inlineStr">
         <is>
           <t>Total Rewards:</t>
         </is>
       </c>
-      <c r="K22" s="74" t="n">
-        <v>516.5</v>
+      <c r="K22" s="73" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="24" ht="20" customHeight="1">
-      <c r="A24" s="71" t="inlineStr">
+      <c r="A24" s="70" t="inlineStr">
         <is>
           <t>APRIL</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="B25" s="72" t="inlineStr">
+      <c r="B25" s="71" t="inlineStr">
         <is>
           <t>Completion:</t>
         </is>
       </c>
-      <c r="D25" s="73" t="inlineStr">
-        <is>
-          <t>24%</t>
-        </is>
-      </c>
-      <c r="H25" s="72" t="inlineStr">
+      <c r="D25" s="72" t="n">
+        <v>0</v>
+      </c>
+      <c r="H25" s="71" t="inlineStr">
         <is>
           <t>Total Rewards:</t>
         </is>
       </c>
-      <c r="K25" s="74" t="n">
-        <v>516.5</v>
+      <c r="K25" s="73" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="27" ht="20" customHeight="1">
-      <c r="A27" s="71" t="inlineStr">
+      <c r="A27" s="70" t="inlineStr">
         <is>
           <t>MAY</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="B28" s="72" t="inlineStr">
+      <c r="B28" s="71" t="inlineStr">
         <is>
           <t>Completion:</t>
         </is>
       </c>
-      <c r="D28" s="73" t="inlineStr">
-        <is>
-          <t>24%</t>
-        </is>
-      </c>
-      <c r="H28" s="72" t="inlineStr">
+      <c r="D28" s="72" t="n">
+        <v>0</v>
+      </c>
+      <c r="H28" s="71" t="inlineStr">
         <is>
           <t>Total Rewards:</t>
         </is>
       </c>
-      <c r="K28" s="74" t="n">
-        <v>516.5</v>
+      <c r="K28" s="73" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="30" ht="20" customHeight="1">
-      <c r="A30" s="71" t="inlineStr">
+      <c r="A30" s="70" t="inlineStr">
         <is>
           <t>JUNE</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="B31" s="72" t="inlineStr">
+      <c r="B31" s="71" t="inlineStr">
         <is>
           <t>Completion:</t>
         </is>
       </c>
-      <c r="D31" s="73" t="inlineStr">
-        <is>
-          <t>24%</t>
-        </is>
-      </c>
-      <c r="H31" s="72" t="inlineStr">
+      <c r="D31" s="72" t="n">
+        <v>0</v>
+      </c>
+      <c r="H31" s="71" t="inlineStr">
         <is>
           <t>Total Rewards:</t>
         </is>
       </c>
-      <c r="K31" s="74" t="n">
-        <v>516.5</v>
+      <c r="K31" s="73" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="33" ht="20" customHeight="1">
-      <c r="A33" s="71" t="inlineStr">
+      <c r="A33" s="70" t="inlineStr">
         <is>
           <t>JULY</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="B34" s="72" t="inlineStr">
+      <c r="B34" s="71" t="inlineStr">
         <is>
           <t>Completion:</t>
         </is>
       </c>
-      <c r="D34" s="73" t="inlineStr">
-        <is>
-          <t>24%</t>
-        </is>
-      </c>
-      <c r="H34" s="72" t="inlineStr">
+      <c r="D34" s="72" t="n">
+        <v>0</v>
+      </c>
+      <c r="H34" s="71" t="inlineStr">
         <is>
           <t>Total Rewards:</t>
         </is>
       </c>
-      <c r="K34" s="74" t="n">
-        <v>516.5</v>
+      <c r="K34" s="73" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="36" ht="20" customHeight="1">
-      <c r="A36" s="71" t="inlineStr">
+      <c r="A36" s="70" t="inlineStr">
         <is>
           <t>AUGUST</t>
         </is>
       </c>
     </row>
     <row r="37">
-      <c r="B37" s="72" t="inlineStr">
+      <c r="B37" s="71" t="inlineStr">
         <is>
           <t>Completion:</t>
         </is>
       </c>
-      <c r="D37" s="73" t="inlineStr">
-        <is>
-          <t>24%</t>
-        </is>
-      </c>
-      <c r="H37" s="72" t="inlineStr">
+      <c r="D37" s="72" t="n">
+        <v>0</v>
+      </c>
+      <c r="H37" s="71" t="inlineStr">
         <is>
           <t>Total Rewards:</t>
         </is>
       </c>
-      <c r="K37" s="74" t="n">
-        <v>516.5</v>
+      <c r="K37" s="73" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="39" ht="20" customHeight="1">
-      <c r="A39" s="71" t="inlineStr">
+      <c r="A39" s="70" t="inlineStr">
         <is>
           <t>SEPTEMBER</t>
         </is>
       </c>
     </row>
     <row r="40">
-      <c r="B40" s="72" t="inlineStr">
+      <c r="B40" s="71" t="inlineStr">
         <is>
           <t>Completion:</t>
         </is>
       </c>
-      <c r="D40" s="73" t="inlineStr">
-        <is>
-          <t>24%</t>
-        </is>
-      </c>
-      <c r="H40" s="72" t="inlineStr">
+      <c r="D40" s="72" t="n">
+        <v>0</v>
+      </c>
+      <c r="H40" s="71" t="inlineStr">
         <is>
           <t>Total Rewards:</t>
         </is>
       </c>
-      <c r="K40" s="74" t="n">
-        <v>516.5</v>
+      <c r="K40" s="73" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="42" ht="20" customHeight="1">
-      <c r="A42" s="71" t="inlineStr">
+      <c r="A42" s="74" t="inlineStr">
         <is>
           <t>OCTOBER</t>
         </is>
       </c>
     </row>
     <row r="43">
-      <c r="B43" s="72" t="inlineStr">
+      <c r="B43" s="71" t="inlineStr">
         <is>
           <t>Completion:</t>
         </is>
       </c>
-      <c r="D43" s="73" t="inlineStr">
-        <is>
-          <t>24%</t>
-        </is>
-      </c>
-      <c r="H43" s="72" t="inlineStr">
+      <c r="D43" s="72">
+        <f>'Monthly habits'!D9</f>
+        <v/>
+      </c>
+      <c r="H43" s="71" t="inlineStr">
         <is>
           <t>Total Rewards:</t>
         </is>
       </c>
-      <c r="K43" s="74" t="n">
-        <v>516.5</v>
+      <c r="K43" s="73">
+        <f>'Monthly habits'!D11</f>
+        <v/>
       </c>
     </row>
     <row r="45" ht="20" customHeight="1">
-      <c r="A45" s="71" t="inlineStr">
+      <c r="A45" s="70" t="inlineStr">
         <is>
           <t>NOVEMBER</t>
         </is>
       </c>
     </row>
     <row r="46">
-      <c r="B46" s="72" t="inlineStr">
+      <c r="B46" s="71" t="inlineStr">
         <is>
           <t>Completion:</t>
         </is>
       </c>
-      <c r="D46" s="73" t="inlineStr">
-        <is>
-          <t>24%</t>
-        </is>
-      </c>
-      <c r="H46" s="72" t="inlineStr">
+      <c r="D46" s="72" t="n">
+        <v>0</v>
+      </c>
+      <c r="H46" s="71" t="inlineStr">
         <is>
           <t>Total Rewards:</t>
         </is>
       </c>
-      <c r="K46" s="74" t="n">
-        <v>516.5</v>
+      <c r="K46" s="73" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="48" ht="20" customHeight="1">
-      <c r="A48" s="71" t="inlineStr">
+      <c r="A48" s="70" t="inlineStr">
         <is>
           <t>DECEMBER</t>
         </is>
       </c>
     </row>
     <row r="49">
-      <c r="B49" s="72" t="inlineStr">
+      <c r="B49" s="71" t="inlineStr">
         <is>
           <t>Completion:</t>
         </is>
       </c>
-      <c r="D49" s="73" t="inlineStr">
-        <is>
-          <t>24%</t>
-        </is>
-      </c>
-      <c r="H49" s="72" t="inlineStr">
+      <c r="D49" s="72" t="n">
+        <v>0</v>
+      </c>
+      <c r="H49" s="71" t="inlineStr">
         <is>
           <t>Total Rewards:</t>
         </is>
       </c>
-      <c r="K49" s="74" t="n">
-        <v>516.5</v>
+      <c r="K49" s="73" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>